<commit_message>
feat: empresas e colaboradores
</commit_message>
<xml_diff>
--- a/analise-marketing/tests/results/abas.xlsx
+++ b/analise-marketing/tests/results/abas.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -426,6 +426,9 @@
       <c r="H1" t="str">
         <v>opt-out</v>
       </c>
+      <c r="I1" t="str">
+        <v>empresas</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -449,17 +452,20 @@
       <c r="G2" t="str">
         <v>E-mail</v>
       </c>
+      <c r="I2" t="str">
+        <v>Aurora</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -486,6 +492,9 @@
       <c r="H1" t="str">
         <v>opt-out</v>
       </c>
+      <c r="I1" t="str">
+        <v>empresas</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -509,10 +518,13 @@
       <c r="G2" t="str">
         <v>WhatsApp</v>
       </c>
+      <c r="I2" t="str">
+        <v>Horizonte</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>